<commit_message>
refactor: update player import templates, repositories, and services for School Demo
</commit_message>
<xml_diff>
--- a/Plantilla_Jugadores_Escuela_Demo.xlsx
+++ b/Plantilla_Jugadores_Escuela_Demo.xlsx
@@ -4,7 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Plantilla Jugadores" sheetId="1" r:id="rId1"/>
-    <sheet name="Instrucciones y Reglas" sheetId="2" r:id="rId2"/>
+    <sheet name="Guia Codigos &amp; Enums" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -398,94 +398,98 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:V21"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="16.83203125" customWidth="1"/>
-    <col min="13" max="13" width="28.83203125" customWidth="1"/>
-    <col min="14" max="14" width="18.83203125" customWidth="1"/>
-    <col min="15" max="15" width="20.83203125" customWidth="1"/>
-    <col min="16" max="16" width="22.83203125" customWidth="1"/>
-    <col min="17" max="17" width="14.83203125" customWidth="1"/>
-    <col min="18" max="18" width="10.83203125" customWidth="1"/>
-    <col min="19" max="19" width="16.83203125" customWidth="1"/>
-    <col min="20" max="20" width="28.83203125" customWidth="1"/>
-    <col min="21" max="21" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="26.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
+    <col min="13" max="13" width="16.83203125" customWidth="1"/>
+    <col min="14" max="14" width="32.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="20.83203125" customWidth="1"/>
+    <col min="17" max="17" width="22.83203125" customWidth="1"/>
+    <col min="18" max="18" width="14.83203125" customWidth="1"/>
+    <col min="19" max="19" width="22.83203125" customWidth="1"/>
+    <col min="20" max="20" width="24.83203125" customWidth="1"/>
+    <col min="21" max="21" width="30.83203125" customWidth="1"/>
+    <col min="22" max="22" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>nombres_jugador</v>
+        <v>nombresJugador</v>
       </c>
       <c r="B1" t="str">
-        <v>apellidos_jugador</v>
+        <v>apellidosJugador</v>
       </c>
       <c r="C1" t="str">
-        <v>tipo_documento_jugador</v>
+        <v>tipoDocumento</v>
       </c>
       <c r="D1" t="str">
-        <v>numero_documento_jugador</v>
+        <v>numeroDocumento</v>
       </c>
       <c r="E1" t="str">
-        <v>fecha_nacimiento_jugador</v>
+        <v>fechaNacimiento</v>
       </c>
       <c r="F1" t="str">
-        <v>genero_jugador</v>
+        <v>genero</v>
       </c>
       <c r="G1" t="str">
-        <v>categoria</v>
+        <v>codigoCategoria</v>
       </c>
       <c r="H1" t="str">
-        <v>posicion_principal</v>
+        <v>nombreCategoria</v>
       </c>
       <c r="I1" t="str">
-        <v>posicion_secundaria</v>
+        <v>posicionPrincipal</v>
       </c>
       <c r="J1" t="str">
-        <v>pierna_habil</v>
+        <v>posicionSecundaria</v>
       </c>
       <c r="K1" t="str">
-        <v>numero_dorsal</v>
+        <v>piernaHabil</v>
       </c>
       <c r="L1" t="str">
+        <v>numeroDorsal</v>
+      </c>
+      <c r="M1" t="str">
         <v>eps</v>
       </c>
-      <c r="M1" t="str">
-        <v>email_jugador</v>
-      </c>
       <c r="N1" t="str">
-        <v>telefono_jugador</v>
+        <v>emailJugador</v>
       </c>
       <c r="O1" t="str">
-        <v>nombres_acudiente</v>
+        <v>telefonoJugador</v>
       </c>
       <c r="P1" t="str">
-        <v>apellidos_acudiente</v>
+        <v>nombresAcudiente</v>
       </c>
       <c r="Q1" t="str">
+        <v>apellidosAcudiente</v>
+      </c>
+      <c r="R1" t="str">
         <v>parentesco</v>
       </c>
-      <c r="R1" t="str">
-        <v>tipo_documento_acudiente</v>
-      </c>
       <c r="S1" t="str">
-        <v>numero_documento_acudiente</v>
+        <v>tipoDocumentoAcudiente</v>
       </c>
       <c r="T1" t="str">
-        <v>email_acudiente</v>
+        <v>numeroDocumentoAcudiente</v>
       </c>
       <c r="U1" t="str">
-        <v>telefono_acudiente</v>
+        <v>emailAcudiente</v>
+      </c>
+      <c r="V1" t="str">
+        <v>telefonoAcudiente</v>
       </c>
     </row>
     <row r="2">
@@ -508,48 +512,51 @@
         <v>MASCULINO</v>
       </c>
       <c r="G2" t="str">
+        <v>CatSub15</v>
+      </c>
+      <c r="H2" t="str">
         <v>Sub-15 Élite A</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>Extremo Izquierdo</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>Delantero Centro</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>DIESTRO</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>11</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>SURA EPS</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>andres.caicedo@escuelademo.com</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>+57 310 555 1101</v>
       </c>
-      <c r="O2" t="str">
+      <c r="P2" t="str">
         <v>Jairo Alberto</v>
       </c>
-      <c r="P2" t="str">
+      <c r="Q2" t="str">
         <v>Caicedo Mina</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="R2" t="str">
         <v>PADRE</v>
       </c>
-      <c r="R2" t="str">
-        <v>CC</v>
-      </c>
       <c r="S2" t="str">
+        <v>CC</v>
+      </c>
+      <c r="T2" t="str">
         <v>71889901</v>
       </c>
-      <c r="T2" t="str">
+      <c r="U2" t="str">
         <v>jairo.caicedo@gmail.com</v>
       </c>
-      <c r="U2" t="str">
+      <c r="V2" t="str">
         <v>+57 311 444 1101</v>
       </c>
     </row>
@@ -573,48 +580,51 @@
         <v>MASCULINO</v>
       </c>
       <c r="G3" t="str">
+        <v>CatSub15</v>
+      </c>
+      <c r="H3" t="str">
         <v>Sub-15 Élite A</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Portero</v>
       </c>
       <c r="I3" t="str">
         <v>Portero</v>
       </c>
       <c r="J3" t="str">
+        <v>Portero</v>
+      </c>
+      <c r="K3" t="str">
         <v>DIESTRO</v>
       </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="L3" t="str">
+      <c r="L3">
+        <v>12</v>
+      </c>
+      <c r="M3" t="str">
         <v>Sanitas EPS</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>santiago.morales@escuelademo.com</v>
       </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
         <v>+57 310 555 1102</v>
       </c>
-      <c r="O3" t="str">
+      <c r="P3" t="str">
         <v>Claudia Patricia</v>
       </c>
-      <c r="P3" t="str">
+      <c r="Q3" t="str">
         <v>Echeverri Zuluaga</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="R3" t="str">
         <v>MADRE</v>
       </c>
-      <c r="R3" t="str">
-        <v>CC</v>
-      </c>
       <c r="S3" t="str">
+        <v>CC</v>
+      </c>
+      <c r="T3" t="str">
         <v>43556677</v>
       </c>
-      <c r="T3" t="str">
+      <c r="U3" t="str">
         <v>claudia.echeverri@gmail.com</v>
       </c>
-      <c r="U3" t="str">
+      <c r="V3" t="str">
         <v>+57 315 777 1102</v>
       </c>
     </row>
@@ -638,49 +648,52 @@
         <v>MASCULINO</v>
       </c>
       <c r="G4" t="str">
+        <v>CatSub15</v>
+      </c>
+      <c r="H4" t="str">
         <v>Sub-15 Élite A</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>Lateral Derecho</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>Defensa Central</v>
       </c>
-      <c r="J4" t="str">
+      <c r="K4" t="str">
         <v>DIESTRO</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>2</v>
       </c>
-      <c r="L4" t="str">
+      <c r="M4" t="str">
         <v>Compensar EPS</v>
       </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
         <v>lucas.restrepo@escuelademo.com</v>
       </c>
-      <c r="N4" t="str">
+      <c r="O4" t="str">
         <v>+57 310 555 1103</v>
       </c>
-      <c r="O4" t="str">
+      <c r="P4" t="str">
         <v>Julián David</v>
       </c>
-      <c r="P4" t="str">
+      <c r="Q4" t="str">
         <v>Restrepo Cardona</v>
       </c>
-      <c r="Q4" t="str">
+      <c r="R4" t="str">
         <v>PADRE</v>
       </c>
-      <c r="R4" t="str">
-        <v>CC</v>
-      </c>
       <c r="S4" t="str">
+        <v>CC</v>
+      </c>
+      <c r="T4" t="str">
         <v>98776655</v>
       </c>
-      <c r="T4" t="str">
+      <c r="U4" t="str">
         <v>julian.restrepo@gmail.com</v>
       </c>
-      <c r="U4" t="str">
-        <v>+57 312 888 1103</v>
+      <c r="V4" t="str">
+        <v>+57 318 888 1103</v>
       </c>
     </row>
     <row r="5">
@@ -697,63 +710,66 @@
         <v>1025890114</v>
       </c>
       <c r="E5" t="str">
-        <v>2012-09-05</v>
+        <v>2011-10-05</v>
       </c>
       <c r="F5" t="str">
         <v>MASCULINO</v>
       </c>
       <c r="G5" t="str">
+        <v>CatSub15</v>
+      </c>
+      <c r="H5" t="str">
         <v>Sub-15 Élite A</v>
       </c>
-      <c r="H5" t="str">
-        <v>Delantero Centro</v>
-      </c>
       <c r="I5" t="str">
-        <v>Extremo Derecho</v>
+        <v>Defensa Central</v>
       </c>
       <c r="J5" t="str">
-        <v>ZURDO</v>
-      </c>
-      <c r="K5">
-        <v>9</v>
-      </c>
-      <c r="L5" t="str">
-        <v>Salud Total EPS</v>
+        <v>Mediocampista Defensivo</v>
+      </c>
+      <c r="K5" t="str">
+        <v>DIESTRO</v>
+      </c>
+      <c r="L5">
+        <v>3</v>
       </c>
       <c r="M5" t="str">
+        <v>SURA EPS</v>
+      </c>
+      <c r="N5" t="str">
         <v>david.quintero@escuelademo.com</v>
       </c>
-      <c r="N5" t="str">
+      <c r="O5" t="str">
         <v>+57 310 555 1104</v>
       </c>
-      <c r="O5" t="str">
+      <c r="P5" t="str">
         <v>Patricia Elena</v>
       </c>
-      <c r="P5" t="str">
+      <c r="Q5" t="str">
         <v>Vega Morales</v>
       </c>
-      <c r="Q5" t="str">
+      <c r="R5" t="str">
         <v>MADRE</v>
       </c>
-      <c r="R5" t="str">
-        <v>CC</v>
-      </c>
       <c r="S5" t="str">
+        <v>CC</v>
+      </c>
+      <c r="T5" t="str">
         <v>52443322</v>
       </c>
-      <c r="T5" t="str">
+      <c r="U5" t="str">
         <v>patricia.vega@gmail.com</v>
       </c>
-      <c r="U5" t="str">
-        <v>+57 314 999 1104</v>
+      <c r="V5" t="str">
+        <v>+57 312 999 1104</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Tomás Alejandro</v>
+        <v>Alejandro</v>
       </c>
       <c r="B6" t="str">
-        <v>Cuervo Londoño</v>
+        <v>Cuervo Restrepo</v>
       </c>
       <c r="C6" t="str">
         <v>TI</v>
@@ -762,63 +778,66 @@
         <v>1025890115</v>
       </c>
       <c r="E6" t="str">
-        <v>2010-04-14</v>
+        <v>2011-12-30</v>
       </c>
       <c r="F6" t="str">
         <v>MASCULINO</v>
       </c>
       <c r="G6" t="str">
-        <v>Sub-17 Nacional Pro</v>
+        <v>CatSub15</v>
       </c>
       <c r="H6" t="str">
-        <v>Volante Defensivo</v>
+        <v>Sub-15 Élite A</v>
       </c>
       <c r="I6" t="str">
+        <v>Mediocampista Defensivo</v>
+      </c>
+      <c r="J6" t="str">
         <v>Defensa Central</v>
       </c>
-      <c r="J6" t="str">
+      <c r="K6" t="str">
         <v>DIESTRO</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>6</v>
       </c>
-      <c r="L6" t="str">
-        <v>Nueva EPS</v>
-      </c>
       <c r="M6" t="str">
-        <v>tomas.cuervo@escuelademo.com</v>
+        <v>Salud Total EPS</v>
       </c>
       <c r="N6" t="str">
+        <v>alejandro.cuervo@escuelademo.com</v>
+      </c>
+      <c r="O6" t="str">
         <v>+57 310 555 1105</v>
       </c>
-      <c r="O6" t="str">
-        <v>Alejandro</v>
-      </c>
       <c r="P6" t="str">
-        <v>Cuervo Restrepo</v>
+        <v>Gonzalo Andrés</v>
       </c>
       <c r="Q6" t="str">
+        <v>Cuervo Londoño</v>
+      </c>
+      <c r="R6" t="str">
         <v>PADRE</v>
       </c>
-      <c r="R6" t="str">
-        <v>CC</v>
-      </c>
       <c r="S6" t="str">
+        <v>CC</v>
+      </c>
+      <c r="T6" t="str">
         <v>70889911</v>
       </c>
-      <c r="T6" t="str">
-        <v>alejandro.cuervo@gmail.com</v>
-      </c>
       <c r="U6" t="str">
-        <v>+57 316 222 1105</v>
+        <v>gonzalo.cuervo@gmail.com</v>
+      </c>
+      <c r="V6" t="str">
+        <v>+57 314 111 1105</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Sebastián</v>
+        <v>Emiliano</v>
       </c>
       <c r="B7" t="str">
-        <v>Arboleda Murillo</v>
+        <v>Toro Zapata</v>
       </c>
       <c r="C7" t="str">
         <v>TI</v>
@@ -827,63 +846,66 @@
         <v>1025890116</v>
       </c>
       <c r="E7" t="str">
-        <v>2010-11-20</v>
+        <v>2011-04-14</v>
       </c>
       <c r="F7" t="str">
         <v>MASCULINO</v>
       </c>
       <c r="G7" t="str">
-        <v>Sub-17 Nacional Pro</v>
+        <v>CatSub15</v>
       </c>
       <c r="H7" t="str">
-        <v>Defensa Central</v>
+        <v>Sub-15 Élite A</v>
       </c>
       <c r="I7" t="str">
-        <v>Lateral Izquierdo</v>
+        <v>Mediocampista Ofensivo</v>
       </c>
       <c r="J7" t="str">
-        <v>AMBIDIESTRO</v>
-      </c>
-      <c r="K7">
-        <v>3</v>
-      </c>
-      <c r="L7" t="str">
-        <v>SURA EPS</v>
+        <v>Extremo Izquierdo</v>
+      </c>
+      <c r="K7" t="str">
+        <v>ZURDO</v>
+      </c>
+      <c r="L7">
+        <v>10</v>
       </c>
       <c r="M7" t="str">
-        <v>sebastian.arboleda@escuelademo.com</v>
+        <v>Nueva EPS</v>
       </c>
       <c r="N7" t="str">
+        <v>emiliano.toro@escuelademo.com</v>
+      </c>
+      <c r="O7" t="str">
         <v>+57 310 555 1106</v>
       </c>
-      <c r="O7" t="str">
-        <v>Fernando</v>
-      </c>
       <c r="P7" t="str">
-        <v>Murillo Caicedo</v>
+        <v>Margarita Rosa</v>
       </c>
       <c r="Q7" t="str">
-        <v>TUTOR_LEGAL</v>
+        <v>Zapata Gómez</v>
       </c>
       <c r="R7" t="str">
-        <v>CC</v>
+        <v>MADRE</v>
       </c>
       <c r="S7" t="str">
-        <v>71334455</v>
+        <v>CC</v>
       </c>
       <c r="T7" t="str">
-        <v>fernando.murillo@gmail.com</v>
+        <v>42998877</v>
       </c>
       <c r="U7" t="str">
-        <v>+57 318 333 1106</v>
+        <v>margarita.zapata@gmail.com</v>
+      </c>
+      <c r="V7" t="str">
+        <v>+57 316 222 1106</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Nicolás</v>
+        <v>Samuel David</v>
       </c>
       <c r="B8" t="str">
-        <v>Bermúdez Castro</v>
+        <v>Henao Beltrán</v>
       </c>
       <c r="C8" t="str">
         <v>TI</v>
@@ -892,128 +914,134 @@
         <v>1025890117</v>
       </c>
       <c r="E8" t="str">
-        <v>2009-06-30</v>
+        <v>2011-09-08</v>
       </c>
       <c r="F8" t="str">
         <v>MASCULINO</v>
       </c>
       <c r="G8" t="str">
-        <v>Sub-17 Nacional Pro</v>
+        <v>CatSub15</v>
       </c>
       <c r="H8" t="str">
+        <v>Sub-15 Élite A</v>
+      </c>
+      <c r="I8" t="str">
         <v>Delantero Centro</v>
       </c>
-      <c r="I8" t="str">
+      <c r="J8" t="str">
         <v>Segundo Delantero</v>
       </c>
-      <c r="J8" t="str">
+      <c r="K8" t="str">
         <v>DIESTRO</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>9</v>
       </c>
-      <c r="L8" t="str">
-        <v>Sanitas EPS</v>
-      </c>
       <c r="M8" t="str">
-        <v>nicolas.bermudez@escuelademo.com</v>
+        <v>Coosalud EPS</v>
       </c>
       <c r="N8" t="str">
+        <v>samuel.henao@escuelademo.com</v>
+      </c>
+      <c r="O8" t="str">
         <v>+57 310 555 1107</v>
       </c>
-      <c r="O8" t="str">
-        <v>Martha Lucía</v>
-      </c>
       <c r="P8" t="str">
-        <v>Castro Ospina</v>
+        <v>Óscar Mauricio</v>
       </c>
       <c r="Q8" t="str">
-        <v>MADRE</v>
+        <v>Henao Peláez</v>
       </c>
       <c r="R8" t="str">
-        <v>CC</v>
+        <v>PADRE</v>
       </c>
       <c r="S8" t="str">
-        <v>32112233</v>
+        <v>CC</v>
       </c>
       <c r="T8" t="str">
-        <v>martha.castro@gmail.com</v>
+        <v>71445566</v>
       </c>
       <c r="U8" t="str">
-        <v>+57 313 111 1107</v>
+        <v>oscar.henao@gmail.com</v>
+      </c>
+      <c r="V8" t="str">
+        <v>+57 317 333 1107</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Juan Pablo</v>
+        <v>Mariana</v>
       </c>
       <c r="B9" t="str">
-        <v>Henao Giraldo</v>
+        <v>Guzmán Osorio</v>
       </c>
       <c r="C9" t="str">
-        <v>CC</v>
+        <v>TI</v>
       </c>
       <c r="D9" t="str">
         <v>1025890118</v>
       </c>
       <c r="E9" t="str">
-        <v>2009-01-15</v>
+        <v>2010-06-19</v>
       </c>
       <c r="F9" t="str">
-        <v>MASCULINO</v>
+        <v>FEMENINO</v>
       </c>
       <c r="G9" t="str">
-        <v>Sub-17 Nacional Pro</v>
+        <v>CatFemSub16</v>
       </c>
       <c r="H9" t="str">
-        <v>Extremo Derecho</v>
+        <v>Femenino Sub-16 Élite</v>
       </c>
       <c r="I9" t="str">
-        <v>Volante Ofensivo</v>
+        <v>Portero</v>
       </c>
       <c r="J9" t="str">
-        <v>ZURDO</v>
-      </c>
-      <c r="K9">
-        <v>7</v>
-      </c>
-      <c r="L9" t="str">
-        <v>Famisanar EPS</v>
+        <v>Portero</v>
+      </c>
+      <c r="K9" t="str">
+        <v>DIESTRO</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
       </c>
       <c r="M9" t="str">
-        <v>juanpablo.henao@escuelademo.com</v>
+        <v>SURA EPS</v>
       </c>
       <c r="N9" t="str">
-        <v>+57 310 555 1108</v>
+        <v>mariana.guzman@escuelademo.com</v>
       </c>
       <c r="O9" t="str">
-        <v>Gabriel Ángel</v>
+        <v>+57 320 666 2201</v>
       </c>
       <c r="P9" t="str">
-        <v>Henao Duque</v>
+        <v>César Augusto</v>
       </c>
       <c r="Q9" t="str">
+        <v>Guzmán Botero</v>
+      </c>
+      <c r="R9" t="str">
         <v>PADRE</v>
       </c>
-      <c r="R9" t="str">
-        <v>CC</v>
-      </c>
       <c r="S9" t="str">
-        <v>15443322</v>
+        <v>CC</v>
       </c>
       <c r="T9" t="str">
-        <v>gabriel.henao@gmail.com</v>
+        <v>71556677</v>
       </c>
       <c r="U9" t="str">
-        <v>+57 300 444 1108</v>
+        <v>cesar.guzman@gmail.com</v>
+      </c>
+      <c r="V9" t="str">
+        <v>+57 321 444 2201</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Emiliano</v>
+        <v>Sara Sofía</v>
       </c>
       <c r="B10" t="str">
-        <v>Vergara Gómez</v>
+        <v>Montoya Arango</v>
       </c>
       <c r="C10" t="str">
         <v>TI</v>
@@ -1022,63 +1050,66 @@
         <v>1025890119</v>
       </c>
       <c r="E10" t="str">
-        <v>2014-05-10</v>
+        <v>2010-02-14</v>
       </c>
       <c r="F10" t="str">
-        <v>MASCULINO</v>
+        <v>FEMENINO</v>
       </c>
       <c r="G10" t="str">
-        <v>Sub-13 Semillero Talentos</v>
+        <v>CatFemSub16</v>
       </c>
       <c r="H10" t="str">
-        <v>Volante Ofensivo</v>
+        <v>Femenino Sub-16 Élite</v>
       </c>
       <c r="I10" t="str">
-        <v>Extremo Izquierdo</v>
+        <v>Defensa Central</v>
       </c>
       <c r="J10" t="str">
-        <v>ZURDO</v>
-      </c>
-      <c r="K10">
-        <v>10</v>
-      </c>
-      <c r="L10" t="str">
-        <v>SURA EPS</v>
+        <v>Lateral Derecho</v>
+      </c>
+      <c r="K10" t="str">
+        <v>DIESTRO</v>
+      </c>
+      <c r="L10">
+        <v>4</v>
       </c>
       <c r="M10" t="str">
-        <v/>
+        <v>Sanitas EPS</v>
       </c>
       <c r="N10" t="str">
-        <v/>
+        <v>sara.montoya@escuelademo.com</v>
       </c>
       <c r="O10" t="str">
-        <v>Lorena</v>
+        <v>+57 320 666 2202</v>
       </c>
       <c r="P10" t="str">
-        <v>Gómez Salcedo</v>
+        <v>Adriana Lucía</v>
       </c>
       <c r="Q10" t="str">
+        <v>Arango Pérez</v>
+      </c>
+      <c r="R10" t="str">
         <v>MADRE</v>
       </c>
-      <c r="R10" t="str">
-        <v>CC</v>
-      </c>
       <c r="S10" t="str">
-        <v>43998877</v>
+        <v>CC</v>
       </c>
       <c r="T10" t="str">
-        <v>lorena.gomez@gmail.com</v>
+        <v>43887766</v>
       </c>
       <c r="U10" t="str">
-        <v>+57 311 555 1109</v>
+        <v>adriana.arango@gmail.com</v>
+      </c>
+      <c r="V10" t="str">
+        <v>+57 322 555 2202</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Matías</v>
+        <v>Valentina</v>
       </c>
       <c r="B11" t="str">
-        <v>Valderrama Palacio</v>
+        <v>Gómez Cárdenas</v>
       </c>
       <c r="C11" t="str">
         <v>TI</v>
@@ -1087,63 +1118,66 @@
         <v>1025890120</v>
       </c>
       <c r="E11" t="str">
-        <v>2014-08-19</v>
+        <v>2010-08-27</v>
       </c>
       <c r="F11" t="str">
-        <v>MASCULINO</v>
+        <v>FEMENINO</v>
       </c>
       <c r="G11" t="str">
-        <v>Sub-13 Semillero Talentos</v>
+        <v>CatFemSub16</v>
       </c>
       <c r="H11" t="str">
-        <v>Portero</v>
+        <v>Femenino Sub-16 Élite</v>
       </c>
       <c r="I11" t="str">
-        <v>Portero</v>
+        <v>Mediocampista Ofensivo</v>
       </c>
       <c r="J11" t="str">
+        <v>Volante Mixto</v>
+      </c>
+      <c r="K11" t="str">
         <v>DIESTRO</v>
       </c>
-      <c r="K11">
-        <v>12</v>
-      </c>
-      <c r="L11" t="str">
+      <c r="L11">
+        <v>10</v>
+      </c>
+      <c r="M11" t="str">
         <v>Compensar EPS</v>
       </c>
-      <c r="M11" t="str">
-        <v/>
-      </c>
       <c r="N11" t="str">
-        <v/>
+        <v>valentina.gomez@escuelademo.com</v>
       </c>
       <c r="O11" t="str">
-        <v>Óscar Iván</v>
+        <v>+57 320 666 2203</v>
       </c>
       <c r="P11" t="str">
-        <v>Valderrama Rúa</v>
+        <v>Héctor Fabio</v>
       </c>
       <c r="Q11" t="str">
+        <v>Gómez Rincón</v>
+      </c>
+      <c r="R11" t="str">
         <v>PADRE</v>
       </c>
-      <c r="R11" t="str">
-        <v>CC</v>
-      </c>
       <c r="S11" t="str">
-        <v>71554433</v>
+        <v>CC</v>
       </c>
       <c r="T11" t="str">
-        <v>oscar.valderrama@gmail.com</v>
+        <v>71667788</v>
       </c>
       <c r="U11" t="str">
-        <v>+57 315 666 1110</v>
+        <v>hector.gomez@gmail.com</v>
+      </c>
+      <c r="V11" t="str">
+        <v>+57 323 666 2203</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Jerónimo</v>
+        <v>Luciana</v>
       </c>
       <c r="B12" t="str">
-        <v>Botero Osorio</v>
+        <v>Bedoya Correa</v>
       </c>
       <c r="C12" t="str">
         <v>TI</v>
@@ -1152,63 +1186,66 @@
         <v>1025890121</v>
       </c>
       <c r="E12" t="str">
-        <v>2013-03-27</v>
+        <v>2010-11-15</v>
       </c>
       <c r="F12" t="str">
-        <v>MASCULINO</v>
+        <v>FEMENINO</v>
       </c>
       <c r="G12" t="str">
-        <v>Sub-13 Semillero Talentos</v>
+        <v>CatFemSub16</v>
       </c>
       <c r="H12" t="str">
-        <v>Lateral Izquierdo</v>
+        <v>Femenino Sub-16 Élite</v>
       </c>
       <c r="I12" t="str">
-        <v>Volante Defensivo</v>
+        <v>Extremo Derecho</v>
       </c>
       <c r="J12" t="str">
-        <v>ZURDO</v>
-      </c>
-      <c r="K12">
-        <v>17</v>
-      </c>
-      <c r="L12" t="str">
-        <v>Coosalud EPS</v>
+        <v>Delantero Centro</v>
+      </c>
+      <c r="K12" t="str">
+        <v>DIESTRO</v>
+      </c>
+      <c r="L12">
+        <v>7</v>
       </c>
       <c r="M12" t="str">
-        <v/>
+        <v>SURA EPS</v>
       </c>
       <c r="N12" t="str">
-        <v/>
+        <v>luciana.bedoya@escuelademo.com</v>
       </c>
       <c r="O12" t="str">
-        <v>Hernán Darío</v>
+        <v>+57 320 666 2204</v>
       </c>
       <c r="P12" t="str">
-        <v>Botero Mejía</v>
+        <v>Luz Dary</v>
       </c>
       <c r="Q12" t="str">
-        <v>ABUELO</v>
+        <v>Correa Gil</v>
       </c>
       <c r="R12" t="str">
-        <v>CC</v>
+        <v>MADRE</v>
       </c>
       <c r="S12" t="str">
-        <v>10223344</v>
+        <v>CC</v>
       </c>
       <c r="T12" t="str">
-        <v>hernan.botero@gmail.com</v>
+        <v>43112233</v>
       </c>
       <c r="U12" t="str">
-        <v>+57 317 777 1111</v>
+        <v>luz.correa@gmail.com</v>
+      </c>
+      <c r="V12" t="str">
+        <v>+57 324 777 2204</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Mariana</v>
+        <v>Camila</v>
       </c>
       <c r="B13" t="str">
-        <v>Salazar Hincapié</v>
+        <v>Vargas Londoño</v>
       </c>
       <c r="C13" t="str">
         <v>TI</v>
@@ -1217,258 +1254,270 @@
         <v>1025890122</v>
       </c>
       <c r="E13" t="str">
-        <v>2011-06-08</v>
+        <v>2010-04-03</v>
       </c>
       <c r="F13" t="str">
         <v>FEMENINO</v>
       </c>
       <c r="G13" t="str">
+        <v>CatFemSub16</v>
+      </c>
+      <c r="H13" t="str">
         <v>Femenino Sub-16 Élite</v>
       </c>
-      <c r="H13" t="str">
+      <c r="I13" t="str">
         <v>Delantero Centro</v>
       </c>
-      <c r="I13" t="str">
-        <v>Extremo Derecho</v>
-      </c>
       <c r="J13" t="str">
-        <v>DIESTRO</v>
-      </c>
-      <c r="K13">
+        <v>Extremo Izquierdo</v>
+      </c>
+      <c r="K13" t="str">
+        <v>ZURDO</v>
+      </c>
+      <c r="L13">
         <v>9</v>
       </c>
-      <c r="L13" t="str">
-        <v>SURA EPS</v>
-      </c>
       <c r="M13" t="str">
-        <v>mariana.salazar@escuelademo.com</v>
+        <v>Nueva EPS</v>
       </c>
       <c r="N13" t="str">
-        <v>+57 310 555 1112</v>
+        <v>camila.vargas@escuelademo.com</v>
       </c>
       <c r="O13" t="str">
-        <v>Beatriz</v>
+        <v>+57 320 666 2205</v>
       </c>
       <c r="P13" t="str">
-        <v>Hincapié Correa</v>
+        <v>Rodrigo</v>
       </c>
       <c r="Q13" t="str">
-        <v>MADRE</v>
+        <v>Vargas Silva</v>
       </c>
       <c r="R13" t="str">
-        <v>CC</v>
+        <v>PADRE</v>
       </c>
       <c r="S13" t="str">
-        <v>32998811</v>
+        <v>CC</v>
       </c>
       <c r="T13" t="str">
-        <v>beatriz.hincapie@gmail.com</v>
+        <v>71778899</v>
       </c>
       <c r="U13" t="str">
-        <v>+57 318 888 1112</v>
+        <v>rodrigo.vargas@gmail.com</v>
+      </c>
+      <c r="V13" t="str">
+        <v>+57 325 888 2205</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Sofía</v>
+        <v>Thiago</v>
       </c>
       <c r="B14" t="str">
-        <v>Cárdenas Beltrán</v>
+        <v>Pineda Carmona</v>
       </c>
       <c r="C14" t="str">
-        <v>TI</v>
+        <v>RC</v>
       </c>
       <c r="D14" t="str">
         <v>1025890123</v>
       </c>
       <c r="E14" t="str">
-        <v>2011-12-14</v>
+        <v>2017-03-20</v>
       </c>
       <c r="F14" t="str">
-        <v>FEMENINO</v>
+        <v>MASCULINO</v>
       </c>
       <c r="G14" t="str">
-        <v>Femenino Sub-16 Élite</v>
+        <v>CatSub9</v>
       </c>
       <c r="H14" t="str">
-        <v>Volante Ofensivo</v>
+        <v>Iniciación Sub-9</v>
       </c>
       <c r="I14" t="str">
-        <v>Volante Defensivo</v>
+        <v>Portero</v>
       </c>
       <c r="J14" t="str">
-        <v>AMBIDIESTRO</v>
-      </c>
-      <c r="K14">
-        <v>8</v>
-      </c>
-      <c r="L14" t="str">
-        <v>Sanitas EPS</v>
+        <v>Portero</v>
+      </c>
+      <c r="K14" t="str">
+        <v>DIESTRO</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
       </c>
       <c r="M14" t="str">
-        <v>sofia.cardenas@escuelademo.com</v>
+        <v>SURA EPS</v>
       </c>
       <c r="N14" t="str">
-        <v>+57 310 555 1113</v>
+        <v/>
       </c>
       <c r="O14" t="str">
+        <v/>
+      </c>
+      <c r="P14" t="str">
         <v>Diego Armando</v>
       </c>
-      <c r="P14" t="str">
-        <v>Cárdenas Arias</v>
-      </c>
       <c r="Q14" t="str">
+        <v>Pineda Marín</v>
+      </c>
+      <c r="R14" t="str">
         <v>PADRE</v>
       </c>
-      <c r="R14" t="str">
-        <v>CC</v>
-      </c>
       <c r="S14" t="str">
-        <v>79223344</v>
+        <v>CC</v>
       </c>
       <c r="T14" t="str">
-        <v>diego.cardenas@gmail.com</v>
+        <v>71990011</v>
       </c>
       <c r="U14" t="str">
-        <v>+57 312 999 1113</v>
+        <v>diego.pineda@gmail.com</v>
+      </c>
+      <c r="V14" t="str">
+        <v>+57 301 333 3301</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Gabriela</v>
+        <v>Matías</v>
       </c>
       <c r="B15" t="str">
-        <v>Moncada Pino</v>
+        <v>Echeverri Ramos</v>
       </c>
       <c r="C15" t="str">
-        <v>TI</v>
+        <v>RC</v>
       </c>
       <c r="D15" t="str">
         <v>1025890124</v>
       </c>
       <c r="E15" t="str">
-        <v>2012-08-01</v>
+        <v>2017-07-11</v>
       </c>
       <c r="F15" t="str">
-        <v>FEMENINO</v>
+        <v>MASCULINO</v>
       </c>
       <c r="G15" t="str">
-        <v>Femenino Sub-16 Élite</v>
+        <v>CatSub9</v>
       </c>
       <c r="H15" t="str">
-        <v>Portero</v>
+        <v>Iniciación Sub-9</v>
       </c>
       <c r="I15" t="str">
-        <v>Portero</v>
+        <v>Defensa Central</v>
       </c>
       <c r="J15" t="str">
+        <v>Lateral Derecho</v>
+      </c>
+      <c r="K15" t="str">
         <v>DIESTRO</v>
       </c>
-      <c r="K15">
-        <v>1</v>
-      </c>
-      <c r="L15" t="str">
-        <v>Nueva EPS</v>
+      <c r="L15">
+        <v>2</v>
       </c>
       <c r="M15" t="str">
-        <v>gabriela.moncada@escuelademo.com</v>
+        <v>Sanitas EPS</v>
       </c>
       <c r="N15" t="str">
-        <v>+57 310 555 1114</v>
+        <v/>
       </c>
       <c r="O15" t="str">
-        <v>Diana Carolina</v>
+        <v/>
       </c>
       <c r="P15" t="str">
-        <v>Pino Vargas</v>
+        <v>Natalia Sofía</v>
       </c>
       <c r="Q15" t="str">
+        <v>Ramos Ortiz</v>
+      </c>
+      <c r="R15" t="str">
         <v>MADRE</v>
       </c>
-      <c r="R15" t="str">
-        <v>CC</v>
-      </c>
       <c r="S15" t="str">
-        <v>52887766</v>
+        <v>CC</v>
       </c>
       <c r="T15" t="str">
-        <v>diana.pino@gmail.com</v>
+        <v>43665544</v>
       </c>
       <c r="U15" t="str">
-        <v>+57 316 111 1114</v>
+        <v>natalia.ramos@gmail.com</v>
+      </c>
+      <c r="V15" t="str">
+        <v>+57 301 444 3302</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Luciana</v>
+        <v>Juan Martín</v>
       </c>
       <c r="B16" t="str">
-        <v>Rincón Duque</v>
+        <v>Suárez Castaño</v>
       </c>
       <c r="C16" t="str">
-        <v>TI</v>
+        <v>RC</v>
       </c>
       <c r="D16" t="str">
         <v>1025890125</v>
       </c>
       <c r="E16" t="str">
-        <v>2010-10-18</v>
+        <v>2017-10-09</v>
       </c>
       <c r="F16" t="str">
-        <v>FEMENINO</v>
+        <v>MASCULINO</v>
       </c>
       <c r="G16" t="str">
-        <v>Femenino Sub-16 Élite</v>
+        <v>CatSub9</v>
       </c>
       <c r="H16" t="str">
-        <v>Defensa Central</v>
+        <v>Iniciación Sub-9</v>
       </c>
       <c r="I16" t="str">
-        <v>Lateral Derecho</v>
+        <v>Mediocampista Ofensivo</v>
       </c>
       <c r="J16" t="str">
+        <v>Delantero Centro</v>
+      </c>
+      <c r="K16" t="str">
         <v>DIESTRO</v>
       </c>
-      <c r="K16">
-        <v>5</v>
-      </c>
-      <c r="L16" t="str">
+      <c r="L16">
+        <v>10</v>
+      </c>
+      <c r="M16" t="str">
         <v>Compensar EPS</v>
       </c>
-      <c r="M16" t="str">
-        <v>luciana.rincon@escuelademo.com</v>
-      </c>
       <c r="N16" t="str">
-        <v>+57 310 555 1115</v>
+        <v/>
       </c>
       <c r="O16" t="str">
-        <v>Roberto Carlos</v>
+        <v/>
       </c>
       <c r="P16" t="str">
-        <v>Rincón Montoya</v>
+        <v>Felipe Andrés</v>
       </c>
       <c r="Q16" t="str">
-        <v>TIO</v>
+        <v>Suárez Villegas</v>
       </c>
       <c r="R16" t="str">
-        <v>CC</v>
+        <v>PADRE</v>
       </c>
       <c r="S16" t="str">
-        <v>80112233</v>
+        <v>CC</v>
       </c>
       <c r="T16" t="str">
-        <v>roberto.rincon@gmail.com</v>
+        <v>71001122</v>
       </c>
       <c r="U16" t="str">
-        <v>+57 319 222 1115</v>
+        <v>felipe.suarez@gmail.com</v>
+      </c>
+      <c r="V16" t="str">
+        <v>+57 301 555 3303</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Thiago Benjamín</v>
+        <v>Dylan</v>
       </c>
       <c r="B17" t="str">
-        <v>Cardona Villa</v>
+        <v>Ochoa Gallego</v>
       </c>
       <c r="C17" t="str">
         <v>RC</v>
@@ -1477,63 +1526,66 @@
         <v>1025890126</v>
       </c>
       <c r="E17" t="str">
-        <v>2018-04-22</v>
+        <v>2018-01-14</v>
       </c>
       <c r="F17" t="str">
         <v>MASCULINO</v>
       </c>
       <c r="G17" t="str">
+        <v>CatSub9</v>
+      </c>
+      <c r="H17" t="str">
         <v>Iniciación Sub-9</v>
-      </c>
-      <c r="H17" t="str">
-        <v>Delantero Centro</v>
       </c>
       <c r="I17" t="str">
         <v>Extremo Derecho</v>
       </c>
       <c r="J17" t="str">
+        <v>Delantero Centro</v>
+      </c>
+      <c r="K17" t="str">
         <v>DIESTRO</v>
       </c>
-      <c r="K17">
+      <c r="L17">
         <v>7</v>
       </c>
-      <c r="L17" t="str">
-        <v>SURA EPS</v>
-      </c>
       <c r="M17" t="str">
-        <v/>
+        <v>Salud Total EPS</v>
       </c>
       <c r="N17" t="str">
         <v/>
       </c>
       <c r="O17" t="str">
-        <v>Daniel Eduardo</v>
+        <v/>
       </c>
       <c r="P17" t="str">
-        <v>Cardona Cano</v>
+        <v>Estefanía</v>
       </c>
       <c r="Q17" t="str">
-        <v>PADRE</v>
+        <v>Gallego Lopera</v>
       </c>
       <c r="R17" t="str">
-        <v>CC</v>
+        <v>MADRE</v>
       </c>
       <c r="S17" t="str">
-        <v>71665544</v>
+        <v>CC</v>
       </c>
       <c r="T17" t="str">
-        <v>daniel.cardona@gmail.com</v>
+        <v>43334455</v>
       </c>
       <c r="U17" t="str">
-        <v>+57 310 333 1116</v>
+        <v>estefania.gallego@gmail.com</v>
+      </c>
+      <c r="V17" t="str">
+        <v>+57 301 666 3304</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Isaac</v>
+        <v>Nicolás</v>
       </c>
       <c r="B18" t="str">
-        <v>Montoya Chaverra</v>
+        <v>Berrío Agudelo</v>
       </c>
       <c r="C18" t="str">
         <v>RC</v>
@@ -1542,128 +1594,134 @@
         <v>1025890127</v>
       </c>
       <c r="E18" t="str">
-        <v>2018-09-11</v>
+        <v>2017-05-28</v>
       </c>
       <c r="F18" t="str">
         <v>MASCULINO</v>
       </c>
       <c r="G18" t="str">
+        <v>CatSub9</v>
+      </c>
+      <c r="H18" t="str">
         <v>Iniciación Sub-9</v>
       </c>
-      <c r="H18" t="str">
-        <v>Volante Ofensivo</v>
-      </c>
       <c r="I18" t="str">
-        <v>Mediocentro Defensivo</v>
+        <v>Delantero Centro</v>
       </c>
       <c r="J18" t="str">
+        <v>Extremo Izquierdo</v>
+      </c>
+      <c r="K18" t="str">
         <v>ZURDO</v>
       </c>
-      <c r="K18">
-        <v>10</v>
-      </c>
-      <c r="L18" t="str">
-        <v>Salud Total EPS</v>
+      <c r="L18">
+        <v>9</v>
       </c>
       <c r="M18" t="str">
-        <v/>
+        <v>Nueva EPS</v>
       </c>
       <c r="N18" t="str">
         <v/>
       </c>
       <c r="O18" t="str">
-        <v>Lina Marcela</v>
+        <v/>
       </c>
       <c r="P18" t="str">
-        <v>Chaverra Lozano</v>
+        <v>Mauricio</v>
       </c>
       <c r="Q18" t="str">
-        <v>MADRE</v>
+        <v>Berrío Castro</v>
       </c>
       <c r="R18" t="str">
-        <v>CC</v>
+        <v>PADRE</v>
       </c>
       <c r="S18" t="str">
-        <v>43112299</v>
+        <v>CC</v>
       </c>
       <c r="T18" t="str">
-        <v>lina.chaverra@gmail.com</v>
+        <v>71112233</v>
       </c>
       <c r="U18" t="str">
-        <v>+57 311 444 1117</v>
+        <v>mauricio.berrio@gmail.com</v>
+      </c>
+      <c r="V18" t="str">
+        <v>+57 301 777 3305</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Maximiliano</v>
+        <v>Brayan Alexis</v>
       </c>
       <c r="B19" t="str">
-        <v>Orozco Serna</v>
+        <v>Mosquera Palacios</v>
       </c>
       <c r="C19" t="str">
-        <v>RC</v>
+        <v>CC</v>
       </c>
       <c r="D19" t="str">
         <v>1025890128</v>
       </c>
       <c r="E19" t="str">
-        <v>2019-02-14</v>
+        <v>2006-08-17</v>
       </c>
       <c r="F19" t="str">
         <v>MASCULINO</v>
       </c>
       <c r="G19" t="str">
-        <v>Iniciación Sub-9</v>
+        <v>CatSub20</v>
       </c>
       <c r="H19" t="str">
-        <v>Portero</v>
+        <v>Sub-20 Proyección Primera</v>
       </c>
       <c r="I19" t="str">
         <v>Portero</v>
       </c>
       <c r="J19" t="str">
+        <v>Portero</v>
+      </c>
+      <c r="K19" t="str">
         <v>DIESTRO</v>
       </c>
-      <c r="K19">
+      <c r="L19">
         <v>1</v>
       </c>
-      <c r="L19" t="str">
-        <v>Sanitas EPS</v>
-      </c>
       <c r="M19" t="str">
-        <v/>
+        <v>SURA EPS</v>
       </c>
       <c r="N19" t="str">
-        <v/>
+        <v>brayan.mosquera@escuelademo.com</v>
       </c>
       <c r="O19" t="str">
-        <v>Andrés Felipe</v>
+        <v>+57 319 777 4401</v>
       </c>
       <c r="P19" t="str">
-        <v>Orozco Marín</v>
+        <v>Eustiquio</v>
       </c>
       <c r="Q19" t="str">
+        <v>Mosquera Rentería</v>
+      </c>
+      <c r="R19" t="str">
         <v>PADRE</v>
       </c>
-      <c r="R19" t="str">
-        <v>CC</v>
-      </c>
       <c r="S19" t="str">
-        <v>98445566</v>
+        <v>CC</v>
       </c>
       <c r="T19" t="str">
-        <v>andres.orozco@gmail.com</v>
+        <v>71223344</v>
       </c>
       <c r="U19" t="str">
-        <v>+57 315 555 1118</v>
+        <v>eustiquio.mosquera@gmail.com</v>
+      </c>
+      <c r="V19" t="str">
+        <v>+57 319 888 4401</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Cristian Camilo</v>
+        <v>Kevin Andrés</v>
       </c>
       <c r="B20" t="str">
-        <v>Palacios Mosquera</v>
+        <v>Castrillón Ruiz</v>
       </c>
       <c r="C20" t="str">
         <v>CC</v>
@@ -1672,63 +1730,66 @@
         <v>1025890129</v>
       </c>
       <c r="E20" t="str">
-        <v>2008-05-19</v>
+        <v>2006-04-12</v>
       </c>
       <c r="F20" t="str">
         <v>MASCULINO</v>
       </c>
       <c r="G20" t="str">
+        <v>CatSub20</v>
+      </c>
+      <c r="H20" t="str">
         <v>Sub-20 Proyección Primera</v>
       </c>
-      <c r="H20" t="str">
+      <c r="I20" t="str">
         <v>Defensa Central</v>
       </c>
-      <c r="I20" t="str">
-        <v>Lateral Derecho</v>
-      </c>
       <c r="J20" t="str">
-        <v>DIESTRO</v>
-      </c>
-      <c r="K20">
-        <v>2</v>
-      </c>
-      <c r="L20" t="str">
-        <v>Nueva EPS</v>
+        <v>Lateral Izquierdo</v>
+      </c>
+      <c r="K20" t="str">
+        <v>ZURDO</v>
+      </c>
+      <c r="L20">
+        <v>3</v>
       </c>
       <c r="M20" t="str">
-        <v>cristian.palacios@escuelademo.com</v>
+        <v>Sanitas EPS</v>
       </c>
       <c r="N20" t="str">
-        <v>+57 310 555 1119</v>
+        <v>kevin.castrillon@escuelademo.com</v>
       </c>
       <c r="O20" t="str">
-        <v>Moisés</v>
+        <v>+57 319 777 4402</v>
       </c>
       <c r="P20" t="str">
-        <v>Palacios Mena</v>
+        <v>Gloria Amparo</v>
       </c>
       <c r="Q20" t="str">
-        <v>PADRE</v>
+        <v>Ruiz Bermúdez</v>
       </c>
       <c r="R20" t="str">
-        <v>CC</v>
+        <v>MADRE</v>
       </c>
       <c r="S20" t="str">
-        <v>11998877</v>
+        <v>CC</v>
       </c>
       <c r="T20" t="str">
-        <v>moises.palacios@gmail.com</v>
+        <v>43778899</v>
       </c>
       <c r="U20" t="str">
-        <v>+57 313 666 1119</v>
+        <v>gloria.ruiz@gmail.com</v>
+      </c>
+      <c r="V20" t="str">
+        <v>+57 319 999 4402</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Brayan Alexis</v>
+        <v>Cristian Camilo</v>
       </c>
       <c r="B21" t="str">
-        <v>Hurtado Mina</v>
+        <v>Vallejo Franco</v>
       </c>
       <c r="C21" t="str">
         <v>CC</v>
@@ -1737,91 +1798,94 @@
         <v>1025890130</v>
       </c>
       <c r="E21" t="str">
-        <v>2008-11-04</v>
+        <v>2007-01-22</v>
       </c>
       <c r="F21" t="str">
         <v>MASCULINO</v>
       </c>
       <c r="G21" t="str">
+        <v>CatSub20</v>
+      </c>
+      <c r="H21" t="str">
         <v>Sub-20 Proyección Primera</v>
-      </c>
-      <c r="H21" t="str">
-        <v>Extremo Izquierdo</v>
       </c>
       <c r="I21" t="str">
         <v>Delantero Centro</v>
       </c>
       <c r="J21" t="str">
-        <v>ZURDO</v>
-      </c>
-      <c r="K21">
-        <v>11</v>
-      </c>
-      <c r="L21" t="str">
-        <v>Emssanar EPS</v>
+        <v>Extremo Derecho</v>
+      </c>
+      <c r="K21" t="str">
+        <v>DIESTRO</v>
+      </c>
+      <c r="L21">
+        <v>9</v>
       </c>
       <c r="M21" t="str">
-        <v>brayan.hurtado@escuelademo.com</v>
+        <v>Compensar EPS</v>
       </c>
       <c r="N21" t="str">
-        <v>+57 310 555 1120</v>
+        <v>cristian.vallejo@escuelademo.com</v>
       </c>
       <c r="O21" t="str">
-        <v>Nubia Stella</v>
+        <v>+57 319 777 4403</v>
       </c>
       <c r="P21" t="str">
-        <v>Mina Quiñones</v>
+        <v>Jaime Alberto</v>
       </c>
       <c r="Q21" t="str">
-        <v>MADRE</v>
+        <v>Vallejo Morales</v>
       </c>
       <c r="R21" t="str">
-        <v>CC</v>
+        <v>PADRE</v>
       </c>
       <c r="S21" t="str">
-        <v>31887766</v>
+        <v>CC</v>
       </c>
       <c r="T21" t="str">
-        <v>nubia.mina@gmail.com</v>
+        <v>71334455</v>
       </c>
       <c r="U21" t="str">
-        <v>+57 317 888 1120</v>
+        <v>jaime.vallejo@gmail.com</v>
+      </c>
+      <c r="V21" t="str">
+        <v>+57 319 111 4403</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V21"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
-    <col min="4" max="4" width="55.83203125" customWidth="1"/>
+    <col min="3" max="3" width="45.83203125" customWidth="1"/>
+    <col min="4" max="4" width="65.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Campo</v>
+        <v>campo</v>
       </c>
       <c r="B1" t="str">
-        <v>Obligatorio</v>
+        <v>obligatorio</v>
       </c>
       <c r="C1" t="str">
-        <v>Formato</v>
+        <v>formato</v>
       </c>
       <c r="D1" t="str">
-        <v>Descripción</v>
+        <v>descripcion</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>nombres_jugador</v>
+        <v>nombresJugador</v>
       </c>
       <c r="B2" t="str">
         <v>SÍ</v>
@@ -1835,7 +1899,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>apellidos_jugador</v>
+        <v>apellidosJugador</v>
       </c>
       <c r="B3" t="str">
         <v>SÍ</v>
@@ -1849,7 +1913,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>tipo_documento_jugador</v>
+        <v>tipoDocumento</v>
       </c>
       <c r="B4" t="str">
         <v>SÍ</v>
@@ -1863,13 +1927,13 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>numero_documento_jugador</v>
+        <v>numeroDocumento</v>
       </c>
       <c r="B5" t="str">
         <v>SÍ</v>
       </c>
       <c r="C5" t="str">
-        <v>Numérico / Alfanumérico único</v>
+        <v>Numérico / Alfanumérico</v>
       </c>
       <c r="D5" t="str">
         <v>Documento sin puntos ni guiones</v>
@@ -1877,7 +1941,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>fecha_nacimiento_jugador</v>
+        <v>fechaNacimiento</v>
       </c>
       <c r="B6" t="str">
         <v>SÍ</v>
@@ -1891,13 +1955,13 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>genero_jugador</v>
+        <v>genero</v>
       </c>
       <c r="B7" t="str">
         <v>NO</v>
       </c>
       <c r="C7" t="str">
-        <v>MASCULINO, FEMENINO, MIXTO</v>
+        <v>MASCULINO, FEMENINO</v>
       </c>
       <c r="D7" t="str">
         <v>Género del atleta</v>
@@ -1905,119 +1969,119 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>categoria</v>
+        <v>codigoCategoria</v>
       </c>
       <c r="B8" t="str">
-        <v>SÍ</v>
+        <v>SÍ (Recomendado)</v>
       </c>
       <c r="C8" t="str">
-        <v>Texto</v>
+        <v>CatSub9, CatSub11, CatSub13, CatSub14, CatSub15, CatSub16, CatSub17, CatSub20, CatFemSub16</v>
       </c>
       <c r="D8" t="str">
-        <v>Si no existe en el club, el sistema la crea automáticamente</v>
+        <v>Código estandarizado para comparación exacta en BD sin errores ortográficos</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>posicion_principal</v>
+        <v>nombreCategoria</v>
       </c>
       <c r="B9" t="str">
         <v>NO</v>
       </c>
       <c r="C9" t="str">
-        <v>Texto</v>
+        <v>Texto Descriptivo</v>
       </c>
       <c r="D9" t="str">
-        <v>Portero, Defensa Central, Volante, Delantero, etc.</v>
+        <v>Nombre visible de la categoría en el sistema (ej: Sub-15 Élite A)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>pierna_habil</v>
+        <v>posicionPrincipal</v>
       </c>
       <c r="B10" t="str">
         <v>NO</v>
       </c>
       <c r="C10" t="str">
-        <v>DIESTRO, ZURDO, AMBIDIESTRO</v>
+        <v>Portero, Defensa Central, Lateral Derecho, Volante, Delantero Centro, etc.</v>
       </c>
       <c r="D10" t="str">
-        <v>Pie dominante</v>
+        <v>Posición táctica principal</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>numero_dorsal</v>
+        <v>piernaHabil</v>
       </c>
       <c r="B11" t="str">
         <v>NO</v>
       </c>
       <c r="C11" t="str">
-        <v>Número entero</v>
+        <v>DIESTRO, ZURDO, AMBIDIESTRO</v>
       </c>
       <c r="D11" t="str">
-        <v>Dorsal en camiseta (debe ser único por categoría)</v>
+        <v>Pie dominante</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>eps</v>
+        <v>numeroDorsal</v>
       </c>
       <c r="B12" t="str">
         <v>NO</v>
       </c>
       <c r="C12" t="str">
-        <v>Texto</v>
+        <v>Número entero (1-99)</v>
       </c>
       <c r="D12" t="str">
-        <v>Entidad de salud médica</v>
+        <v>Dorsal en camiseta (único por categoría)</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>email_jugador</v>
+        <v>eps</v>
       </c>
       <c r="B13" t="str">
-        <v>Opcional (SÍ si &gt;= 14)</v>
+        <v>NO</v>
       </c>
       <c r="C13" t="str">
-        <v>Email válido</v>
+        <v>Texto</v>
       </c>
       <c r="D13" t="str">
-        <v>Para login del jugador al portal/app</v>
+        <v>Entidad de salud médica</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>telefono_jugador</v>
+        <v>emailJugador</v>
       </c>
       <c r="B14" t="str">
-        <v>NO</v>
+        <v>Opcional (SÍ si &gt;= 14)</v>
       </c>
       <c r="C14" t="str">
-        <v>Teléfono</v>
+        <v>Email válido</v>
       </c>
       <c r="D14" t="str">
-        <v>Número de WhatsApp/móvil</v>
+        <v>Para login del jugador al portal/app</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>nombres_acudiente</v>
+        <v>telefonoJugador</v>
       </c>
       <c r="B15" t="str">
-        <v>SÍ para menores</v>
+        <v>NO</v>
       </c>
       <c r="C15" t="str">
-        <v>Texto</v>
+        <v>Teléfono</v>
       </c>
       <c r="D15" t="str">
-        <v>Nombre del padre, madre o tutor legal</v>
+        <v>Número de WhatsApp/móvil</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>apellidos_acudiente</v>
+        <v>nombresAcudiente</v>
       </c>
       <c r="B16" t="str">
         <v>SÍ para menores</v>
@@ -2026,82 +2090,96 @@
         <v>Texto</v>
       </c>
       <c r="D16" t="str">
-        <v>Apellidos del acudiente</v>
+        <v>Nombre del padre, madre o tutor legal</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>parentesco</v>
+        <v>apellidosAcudiente</v>
       </c>
       <c r="B17" t="str">
-        <v>SÍ</v>
+        <v>SÍ para menores</v>
       </c>
       <c r="C17" t="str">
-        <v>PADRE, MADRE, TUTOR_LEGAL, ABUELO, TIO</v>
+        <v>Texto</v>
       </c>
       <c r="D17" t="str">
-        <v>Parentesco con el atleta</v>
+        <v>Apellidos del acudiente</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>tipo_documento_acudiente</v>
+        <v>parentesco</v>
       </c>
       <c r="B18" t="str">
         <v>SÍ</v>
       </c>
       <c r="C18" t="str">
-        <v>CC, CE, PASAPORTE, PEP</v>
+        <v>PADRE, MADRE, TUTOR_LEGAL, OTRO</v>
       </c>
       <c r="D18" t="str">
-        <v>Tipo de documento del acudiente</v>
+        <v>Parentesco con el atleta</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>numero_documento_acudiente</v>
+        <v>tipoDocumentoAcudiente</v>
       </c>
       <c r="B19" t="str">
         <v>SÍ</v>
       </c>
       <c r="C19" t="str">
-        <v>Numérico</v>
+        <v>CC, CE, PASAPORTE, PEP</v>
       </c>
       <c r="D19" t="str">
-        <v>Cédula del acudiente</v>
+        <v>Tipo de documento del acudiente</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>email_acudiente</v>
+        <v>numeroDocumentoAcudiente</v>
       </c>
       <c r="B20" t="str">
         <v>SÍ</v>
       </c>
       <c r="C20" t="str">
-        <v>Email válido</v>
+        <v>Numérico</v>
       </c>
       <c r="D20" t="str">
-        <v>Para login del padre al portal de pagos y boletines</v>
+        <v>Cédula del acudiente</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>telefono_acudiente</v>
+        <v>emailAcudiente</v>
       </c>
       <c r="B21" t="str">
         <v>SÍ</v>
       </c>
       <c r="C21" t="str">
+        <v>Email válido</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Para login del padre al portal de pagos y seguimiento</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>telefonoAcudiente</v>
+      </c>
+      <c r="B22" t="str">
+        <v>SÍ</v>
+      </c>
+      <c r="C22" t="str">
         <v>Teléfono</v>
       </c>
-      <c r="D21" t="str">
+      <c r="D22" t="str">
         <v>Notificaciones WhatsApp</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>